<commit_message>
Add CLI refresh flag
</commit_message>
<xml_diff>
--- a/data/sp500_raw_data.xlsx
+++ b/data/sp500_raw_data.xlsx
@@ -181,10 +181,10 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Refreshed from Yahoo Finance 500.PA history and the Amundi LU1681048804 factsheet on 2026-03-10 17:06:20
-https://finance.yahoo.com/quote/500.PA/history
-https://www.amundietf.lu/pdfDocuments/monthly-factsheet/LU1681048804/ENG/LUX/RETAIL/ETF
-Earliest authoritative month available for this series: 2010-06-01.</t>
+        <t>Refreshed from Yahoo Finance 500.PA monthly history and the Amundi LU1681048804 factsheet on 2026-03-10 23:18:04.
+https://finance.yahoo.com/quote/500.PA/history/
+https://www.amundietf.lu/en/individual/products/equity/amundi-sp-500-swap-ucits-etf-eur-acc/lu1681048804
+Earliest reliable live month for this series: 2010-06-01.</t>
       </text>
     </comment>
   </commentList>

</xml_diff>

<commit_message>
Update sp500 raw data file
</commit_message>
<xml_diff>
--- a/data/sp500_raw_data.xlsx
+++ b/data/sp500_raw_data.xlsx
@@ -181,7 +181,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Refreshed from Yahoo Finance 500.PA monthly history and the Amundi LU1681048804 factsheet on 2026-03-11 00:03:09.
+        <t>Refreshed from Yahoo Finance 500.PA monthly history on 2026-03-11 01:25:13.
 https://finance.yahoo.com/quote/500.PA/history/
 https://www.amundietf.lu/en/individual/products/equity/amundi-sp-500-swap-ucits-etf-eur-acc/lu1681048804
 Earliest reliable live month for this series: 2010-06-01.</t>
@@ -391,7 +391,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1000"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">

</xml_diff>